<commit_message>
Add github repo link file
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mepra\Desktop\IT23272736-ITPM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F4E289-72D1-4A31-A26A-9B2518C8F09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E116B708-E058-444D-8339-D2DFBC9D323F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1104,22 +1104,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1404,7 +1404,7 @@
   <dimension ref="A1:H201"/>
   <sheetFormatPr defaultRowHeight="49.95" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.109375" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="16.5546875" customWidth="1"/>
     <col min="3" max="3" width="33.5546875" customWidth="1"/>
     <col min="4" max="4" width="29.77734375" customWidth="1"/>
@@ -1442,28 +1442,28 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="F2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="7" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1498,28 +1498,28 @@
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="2" t="s">
+      <c r="F6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="7" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1554,28 +1554,28 @@
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="F10" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="8" t="s">
+      <c r="F10" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="7" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1610,28 +1610,28 @@
       <c r="H13" s="4"/>
     </row>
     <row r="14" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="2" t="s">
+      <c r="F14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1666,28 +1666,28 @@
       <c r="H17" s="4"/>
     </row>
     <row r="18" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="2" t="s">
+      <c r="F18" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="8" t="s">
+      <c r="H18" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1722,28 +1722,28 @@
       <c r="H21" s="4"/>
     </row>
     <row r="22" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="2" t="s">
+      <c r="F22" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="H22" s="8" t="s">
+      <c r="H22" s="7" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1778,28 +1778,28 @@
       <c r="H25" s="4"/>
     </row>
     <row r="26" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="F26" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G26" s="2" t="s">
+      <c r="F26" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H26" s="8" t="s">
+      <c r="H26" s="7" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1834,28 +1834,28 @@
       <c r="H29" s="4"/>
     </row>
     <row r="30" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="F30" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G30" s="2" t="s">
+      <c r="F30" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H30" s="8" t="s">
+      <c r="H30" s="7" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1890,28 +1890,28 @@
       <c r="H33" s="4"/>
     </row>
     <row r="34" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="F34" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G34" s="2" t="s">
+      <c r="F34" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="H34" s="8" t="s">
+      <c r="H34" s="7" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1946,28 +1946,28 @@
       <c r="H37" s="4"/>
     </row>
     <row r="38" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E38" s="7" t="s">
+      <c r="E38" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="F38" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G38" s="2" t="s">
+      <c r="F38" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H38" s="8" t="s">
+      <c r="H38" s="7" t="s">
         <v>58</v>
       </c>
     </row>
@@ -2002,28 +2002,28 @@
       <c r="H41" s="4"/>
     </row>
     <row r="42" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="6" t="s">
+      <c r="A42" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E42" s="7" t="s">
+      <c r="E42" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="F42" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G42" s="2" t="s">
+      <c r="F42" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H42" s="8" t="s">
+      <c r="H42" s="7" t="s">
         <v>63</v>
       </c>
     </row>
@@ -2058,28 +2058,28 @@
       <c r="H45" s="4"/>
     </row>
     <row r="46" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="6" t="s">
+      <c r="A46" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E46" s="7" t="s">
+      <c r="E46" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="F46" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G46" s="2" t="s">
+      <c r="F46" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H46" s="8" t="s">
+      <c r="H46" s="7" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2114,28 +2114,28 @@
       <c r="H49" s="4"/>
     </row>
     <row r="50" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C50" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D50" s="7" t="s">
+      <c r="D50" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="E50" s="7" t="s">
+      <c r="E50" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="F50" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G50" s="2" t="s">
+      <c r="F50" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G50" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="H50" s="8" t="s">
+      <c r="H50" s="7" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2170,28 +2170,28 @@
       <c r="H53" s="4"/>
     </row>
     <row r="54" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="D54" s="7" t="s">
+      <c r="D54" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E54" s="7" t="s">
+      <c r="E54" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="F54" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G54" s="2" t="s">
+      <c r="F54" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G54" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="H54" s="8" t="s">
+      <c r="H54" s="7" t="s">
         <v>77</v>
       </c>
     </row>
@@ -2226,28 +2226,28 @@
       <c r="H57" s="4"/>
     </row>
     <row r="58" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="6" t="s">
+      <c r="A58" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="C58" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="D58" s="7" t="s">
+      <c r="D58" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E58" s="7" t="s">
+      <c r="E58" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="F58" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G58" s="2" t="s">
+      <c r="F58" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G58" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="H58" s="8" t="s">
+      <c r="H58" s="7" t="s">
         <v>82</v>
       </c>
     </row>
@@ -2282,28 +2282,28 @@
       <c r="H61" s="4"/>
     </row>
     <row r="62" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="6" t="s">
+      <c r="A62" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C62" s="5" t="s">
+      <c r="C62" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D62" s="7" t="s">
+      <c r="D62" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="E62" s="7" t="s">
+      <c r="E62" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="F62" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G62" s="2" t="s">
+      <c r="F62" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G62" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="H62" s="8" t="s">
+      <c r="H62" s="7" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2338,28 +2338,28 @@
       <c r="H65" s="4"/>
     </row>
     <row r="66" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="6" t="s">
+      <c r="A66" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C66" s="5" t="s">
+      <c r="C66" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D66" s="7" t="s">
+      <c r="D66" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="E66" s="7" t="s">
+      <c r="E66" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="F66" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G66" s="2" t="s">
+      <c r="F66" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G66" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="H66" s="8" t="s">
+      <c r="H66" s="7" t="s">
         <v>92</v>
       </c>
     </row>
@@ -2394,28 +2394,28 @@
       <c r="H69" s="4"/>
     </row>
     <row r="70" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="6" t="s">
+      <c r="A70" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C70" s="5" t="s">
+      <c r="C70" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="D70" s="7" t="s">
+      <c r="D70" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="E70" s="7" t="s">
+      <c r="E70" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="F70" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G70" s="2" t="s">
+      <c r="F70" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G70" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H70" s="8" t="s">
+      <c r="H70" s="7" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2450,28 +2450,28 @@
       <c r="H73" s="4"/>
     </row>
     <row r="74" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="6" t="s">
+      <c r="A74" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C74" s="5" t="s">
+      <c r="C74" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="D74" s="7" t="s">
+      <c r="D74" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E74" s="7" t="s">
+      <c r="E74" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="F74" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G74" s="2" t="s">
+      <c r="F74" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G74" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="H74" s="8" t="s">
+      <c r="H74" s="7" t="s">
         <v>100</v>
       </c>
     </row>
@@ -2506,28 +2506,28 @@
       <c r="H77" s="4"/>
     </row>
     <row r="78" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="6" t="s">
+      <c r="A78" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C78" s="5" t="s">
+      <c r="C78" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D78" s="7" t="s">
+      <c r="D78" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E78" s="7" t="s">
+      <c r="E78" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="F78" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G78" s="2" t="s">
+      <c r="F78" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G78" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="H78" s="8" t="s">
+      <c r="H78" s="7" t="s">
         <v>105</v>
       </c>
     </row>
@@ -2562,28 +2562,28 @@
       <c r="H81" s="4"/>
     </row>
     <row r="82" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="6" t="s">
+      <c r="A82" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C82" s="5" t="s">
+      <c r="C82" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D82" s="7" t="s">
+      <c r="D82" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="E82" s="7" t="s">
+      <c r="E82" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="F82" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G82" s="2" t="s">
+      <c r="F82" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G82" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H82" s="8" t="s">
+      <c r="H82" s="7" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2618,28 +2618,28 @@
       <c r="H85" s="4"/>
     </row>
     <row r="86" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="6" t="s">
+      <c r="A86" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B86" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C86" s="5" t="s">
+      <c r="C86" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="D86" s="7" t="s">
+      <c r="D86" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="E86" s="7" t="s">
+      <c r="E86" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="F86" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G86" s="2" t="s">
+      <c r="F86" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G86" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="H86" s="8" t="s">
+      <c r="H86" s="7" t="s">
         <v>114</v>
       </c>
     </row>
@@ -2674,28 +2674,28 @@
       <c r="H89" s="4"/>
     </row>
     <row r="90" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="6" t="s">
+      <c r="A90" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B90" s="2" t="s">
+      <c r="B90" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C90" s="5" t="s">
+      <c r="C90" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="D90" s="7" t="s">
+      <c r="D90" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E90" s="7" t="s">
+      <c r="E90" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="F90" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G90" s="2" t="s">
+      <c r="F90" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G90" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H90" s="8" t="s">
+      <c r="H90" s="7" t="s">
         <v>118</v>
       </c>
     </row>
@@ -2730,28 +2730,28 @@
       <c r="H93" s="4"/>
     </row>
     <row r="94" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="6" t="s">
+      <c r="A94" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B94" s="2" t="s">
+      <c r="B94" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C94" s="5" t="s">
+      <c r="C94" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="D94" s="7" t="s">
+      <c r="D94" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="E94" s="7" t="s">
+      <c r="E94" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="F94" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G94" s="2" t="s">
+      <c r="F94" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G94" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H94" s="8" t="s">
+      <c r="H94" s="7" t="s">
         <v>123</v>
       </c>
     </row>
@@ -2786,28 +2786,28 @@
       <c r="H97" s="4"/>
     </row>
     <row r="98" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="6" t="s">
+      <c r="A98" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="B98" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C98" s="5" t="s">
+      <c r="C98" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="D98" s="7" t="s">
+      <c r="D98" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="E98" s="7" t="s">
+      <c r="E98" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="F98" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G98" s="2" t="s">
+      <c r="F98" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G98" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="H98" s="8" t="s">
+      <c r="H98" s="7" t="s">
         <v>128</v>
       </c>
     </row>
@@ -2842,28 +2842,28 @@
       <c r="H101" s="4"/>
     </row>
     <row r="102" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="6" t="s">
+      <c r="A102" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B102" s="2" t="s">
+      <c r="B102" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C102" s="5" t="s">
+      <c r="C102" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="D102" s="7" t="s">
+      <c r="D102" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="E102" s="7" t="s">
+      <c r="E102" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="F102" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G102" s="2" t="s">
+      <c r="F102" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G102" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="H102" s="8" t="s">
+      <c r="H102" s="7" t="s">
         <v>132</v>
       </c>
     </row>
@@ -2898,28 +2898,28 @@
       <c r="H105" s="4"/>
     </row>
     <row r="106" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="6" t="s">
+      <c r="A106" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B106" s="2" t="s">
+      <c r="B106" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C106" s="5" t="s">
+      <c r="C106" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="D106" s="7" t="s">
+      <c r="D106" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="E106" s="7" t="s">
+      <c r="E106" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="F106" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G106" s="2" t="s">
+      <c r="F106" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G106" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="H106" s="8" t="s">
+      <c r="H106" s="7" t="s">
         <v>137</v>
       </c>
     </row>
@@ -2954,28 +2954,28 @@
       <c r="H109" s="4"/>
     </row>
     <row r="110" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="6" t="s">
+      <c r="A110" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B110" s="2" t="s">
+      <c r="B110" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C110" s="5" t="s">
+      <c r="C110" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="D110" s="7" t="s">
+      <c r="D110" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="E110" s="7" t="s">
+      <c r="E110" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="F110" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G110" s="2" t="s">
+      <c r="F110" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G110" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H110" s="8" t="s">
+      <c r="H110" s="7" t="s">
         <v>141</v>
       </c>
     </row>
@@ -3010,28 +3010,28 @@
       <c r="H113" s="4"/>
     </row>
     <row r="114" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="6" t="s">
+      <c r="A114" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B114" s="2" t="s">
+      <c r="B114" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C114" s="5" t="s">
+      <c r="C114" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="D114" s="7" t="s">
+      <c r="D114" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="E114" s="7" t="s">
+      <c r="E114" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="F114" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G114" s="2" t="s">
+      <c r="F114" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G114" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="H114" s="8" t="s">
+      <c r="H114" s="7" t="s">
         <v>146</v>
       </c>
     </row>
@@ -3066,28 +3066,28 @@
       <c r="H117" s="4"/>
     </row>
     <row r="118" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="6" t="s">
+      <c r="A118" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B118" s="2" t="s">
+      <c r="B118" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C118" s="5" t="s">
+      <c r="C118" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="D118" s="7" t="s">
+      <c r="D118" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="E118" s="7" t="s">
+      <c r="E118" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="F118" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G118" s="2" t="s">
+      <c r="F118" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G118" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="H118" s="8" t="s">
+      <c r="H118" s="7" t="s">
         <v>151</v>
       </c>
     </row>
@@ -3122,28 +3122,28 @@
       <c r="H121" s="4"/>
     </row>
     <row r="122" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="6" t="s">
+      <c r="A122" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B122" s="2" t="s">
+      <c r="B122" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C122" s="5" t="s">
+      <c r="C122" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="D122" s="7" t="s">
+      <c r="D122" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="E122" s="7" t="s">
+      <c r="E122" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="F122" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G122" s="2" t="s">
+      <c r="F122" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G122" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="H122" s="8" t="s">
+      <c r="H122" s="7" t="s">
         <v>156</v>
       </c>
     </row>
@@ -3178,28 +3178,28 @@
       <c r="H125" s="4"/>
     </row>
     <row r="126" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="6" t="s">
+      <c r="A126" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B126" s="2" t="s">
+      <c r="B126" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C126" s="5" t="s">
+      <c r="C126" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="D126" s="7" t="s">
+      <c r="D126" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="E126" s="7" t="s">
+      <c r="E126" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="F126" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G126" s="2" t="s">
+      <c r="F126" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G126" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H126" s="8" t="s">
+      <c r="H126" s="7" t="s">
         <v>161</v>
       </c>
     </row>
@@ -3234,28 +3234,28 @@
       <c r="H129" s="4"/>
     </row>
     <row r="130" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="6" t="s">
+      <c r="A130" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B130" s="2" t="s">
+      <c r="B130" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C130" s="5" t="s">
+      <c r="C130" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="D130" s="7" t="s">
+      <c r="D130" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="E130" s="7" t="s">
+      <c r="E130" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="F130" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G130" s="2" t="s">
+      <c r="F130" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G130" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="H130" s="8" t="s">
+      <c r="H130" s="7" t="s">
         <v>166</v>
       </c>
     </row>
@@ -3290,28 +3290,28 @@
       <c r="H133" s="4"/>
     </row>
     <row r="134" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="6" t="s">
+      <c r="A134" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="B134" s="2" t="s">
+      <c r="B134" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C134" s="5" t="s">
+      <c r="C134" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="D134" s="7" t="s">
+      <c r="D134" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="E134" s="7" t="s">
+      <c r="E134" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="F134" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G134" s="2" t="s">
+      <c r="F134" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G134" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="H134" s="8" t="s">
+      <c r="H134" s="7" t="s">
         <v>171</v>
       </c>
     </row>
@@ -3346,28 +3346,28 @@
       <c r="H137" s="4"/>
     </row>
     <row r="138" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="6" t="s">
+      <c r="A138" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="B138" s="2" t="s">
+      <c r="B138" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C138" s="5" t="s">
+      <c r="C138" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="D138" s="7" t="s">
+      <c r="D138" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="E138" s="7" t="s">
+      <c r="E138" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="F138" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G138" s="2" t="s">
+      <c r="F138" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G138" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="H138" s="8" t="s">
+      <c r="H138" s="7" t="s">
         <v>176</v>
       </c>
     </row>
@@ -3402,28 +3402,28 @@
       <c r="H141" s="4"/>
     </row>
     <row r="142" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A142" s="6" t="s">
+      <c r="A142" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B142" s="2" t="s">
+      <c r="B142" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C142" s="5" t="s">
+      <c r="C142" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="D142" s="7" t="s">
+      <c r="D142" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="E142" s="7" t="s">
+      <c r="E142" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="F142" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G142" s="2" t="s">
+      <c r="F142" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G142" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="H142" s="8" t="s">
+      <c r="H142" s="7" t="s">
         <v>181</v>
       </c>
     </row>
@@ -3458,28 +3458,28 @@
       <c r="H145" s="4"/>
     </row>
     <row r="146" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="6" t="s">
+      <c r="A146" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B146" s="2" t="s">
+      <c r="B146" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C146" s="5" t="s">
+      <c r="C146" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="D146" s="7" t="s">
+      <c r="D146" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="E146" s="7" t="s">
+      <c r="E146" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="F146" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G146" s="2" t="s">
+      <c r="F146" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G146" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="H146" s="8" t="s">
+      <c r="H146" s="7" t="s">
         <v>186</v>
       </c>
     </row>
@@ -3514,28 +3514,28 @@
       <c r="H149" s="4"/>
     </row>
     <row r="150" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="6" t="s">
+      <c r="A150" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="B150" s="2" t="s">
+      <c r="B150" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C150" s="5" t="s">
+      <c r="C150" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="D150" s="7" t="s">
+      <c r="D150" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="E150" s="7" t="s">
+      <c r="E150" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="F150" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G150" s="2" t="s">
+      <c r="F150" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G150" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="H150" s="8" t="s">
+      <c r="H150" s="7" t="s">
         <v>191</v>
       </c>
     </row>
@@ -3570,28 +3570,28 @@
       <c r="H153" s="4"/>
     </row>
     <row r="154" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="6" t="s">
+      <c r="A154" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="B154" s="2" t="s">
+      <c r="B154" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C154" s="5" t="s">
+      <c r="C154" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="D154" s="7" t="s">
+      <c r="D154" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="E154" s="7" t="s">
+      <c r="E154" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="F154" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G154" s="2" t="s">
+      <c r="F154" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G154" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="H154" s="8" t="s">
+      <c r="H154" s="7" t="s">
         <v>196</v>
       </c>
     </row>
@@ -3626,28 +3626,28 @@
       <c r="H157" s="4"/>
     </row>
     <row r="158" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A158" s="6" t="s">
+      <c r="A158" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B158" s="2" t="s">
+      <c r="B158" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C158" s="5" t="s">
+      <c r="C158" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="D158" s="7" t="s">
+      <c r="D158" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="E158" s="7" t="s">
+      <c r="E158" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="F158" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G158" s="2" t="s">
+      <c r="F158" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G158" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="H158" s="8" t="s">
+      <c r="H158" s="7" t="s">
         <v>201</v>
       </c>
     </row>
@@ -3682,28 +3682,28 @@
       <c r="H161" s="4"/>
     </row>
     <row r="162" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="6" t="s">
+      <c r="A162" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="B162" s="2" t="s">
+      <c r="B162" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C162" s="5" t="s">
+      <c r="C162" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="D162" s="7" t="s">
+      <c r="D162" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="E162" s="7" t="s">
+      <c r="E162" s="5" t="s">
         <v>285</v>
       </c>
-      <c r="F162" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G162" s="2" t="s">
+      <c r="F162" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G162" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="H162" s="8" t="s">
+      <c r="H162" s="7" t="s">
         <v>206</v>
       </c>
     </row>
@@ -3738,28 +3738,28 @@
       <c r="H165" s="4"/>
     </row>
     <row r="166" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A166" s="6" t="s">
+      <c r="A166" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="B166" s="2" t="s">
+      <c r="B166" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C166" s="5" t="s">
+      <c r="C166" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="D166" s="7" t="s">
+      <c r="D166" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="E166" s="7" t="s">
+      <c r="E166" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="F166" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G166" s="2" t="s">
+      <c r="F166" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G166" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="H166" s="8" t="s">
+      <c r="H166" s="7" t="s">
         <v>211</v>
       </c>
     </row>
@@ -3794,28 +3794,28 @@
       <c r="H169" s="4"/>
     </row>
     <row r="170" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A170" s="6" t="s">
+      <c r="A170" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B170" s="2" t="s">
+      <c r="B170" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C170" s="5" t="s">
+      <c r="C170" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="D170" s="7" t="s">
+      <c r="D170" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="E170" s="7" t="s">
+      <c r="E170" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="F170" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G170" s="2" t="s">
+      <c r="F170" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G170" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="H170" s="8" t="s">
+      <c r="H170" s="7" t="s">
         <v>216</v>
       </c>
     </row>
@@ -3850,28 +3850,28 @@
       <c r="H173" s="4"/>
     </row>
     <row r="174" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A174" s="6" t="s">
+      <c r="A174" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B174" s="2" t="s">
+      <c r="B174" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C174" s="5" t="s">
+      <c r="C174" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="D174" s="7" t="s">
+      <c r="D174" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="E174" s="7" t="s">
+      <c r="E174" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="F174" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G174" s="2" t="s">
+      <c r="F174" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G174" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="H174" s="8" t="s">
+      <c r="H174" s="7" t="s">
         <v>221</v>
       </c>
     </row>
@@ -3906,28 +3906,28 @@
       <c r="H177" s="4"/>
     </row>
     <row r="178" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A178" s="6" t="s">
+      <c r="A178" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B178" s="2" t="s">
+      <c r="B178" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C178" s="5" t="s">
+      <c r="C178" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="D178" s="7" t="s">
+      <c r="D178" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="E178" s="7" t="s">
+      <c r="E178" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="F178" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G178" s="2" t="s">
+      <c r="F178" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G178" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="H178" s="8" t="s">
+      <c r="H178" s="7" t="s">
         <v>226</v>
       </c>
     </row>
@@ -3962,28 +3962,28 @@
       <c r="H181" s="4"/>
     </row>
     <row r="182" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A182" s="6" t="s">
+      <c r="A182" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B182" s="2" t="s">
+      <c r="B182" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C182" s="5" t="s">
+      <c r="C182" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="D182" s="7" t="s">
+      <c r="D182" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="E182" s="7" t="s">
+      <c r="E182" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="F182" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G182" s="2" t="s">
+      <c r="F182" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G182" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="H182" s="8" t="s">
+      <c r="H182" s="7" t="s">
         <v>231</v>
       </c>
     </row>
@@ -4018,28 +4018,28 @@
       <c r="H185" s="4"/>
     </row>
     <row r="186" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A186" s="6" t="s">
+      <c r="A186" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B186" s="2" t="s">
+      <c r="B186" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C186" s="5" t="s">
+      <c r="C186" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="D186" s="7" t="s">
+      <c r="D186" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="E186" s="7" t="s">
+      <c r="E186" s="5" t="s">
         <v>289</v>
       </c>
-      <c r="F186" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G186" s="2" t="s">
+      <c r="F186" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G186" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="H186" s="8" t="s">
+      <c r="H186" s="7" t="s">
         <v>236</v>
       </c>
     </row>
@@ -4074,28 +4074,28 @@
       <c r="H189" s="4"/>
     </row>
     <row r="190" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A190" s="6" t="s">
+      <c r="A190" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="B190" s="2" t="s">
+      <c r="B190" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C190" s="5" t="s">
+      <c r="C190" s="8" t="s">
         <v>238</v>
       </c>
-      <c r="D190" s="7" t="s">
+      <c r="D190" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="E190" s="7" t="s">
+      <c r="E190" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="F190" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G190" s="2" t="s">
+      <c r="F190" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G190" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="H190" s="8" t="s">
+      <c r="H190" s="7" t="s">
         <v>241</v>
       </c>
     </row>
@@ -4130,28 +4130,28 @@
       <c r="H193" s="4"/>
     </row>
     <row r="194" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A194" s="6" t="s">
+      <c r="A194" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="B194" s="2" t="s">
+      <c r="B194" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C194" s="5" t="s">
+      <c r="C194" s="8" t="s">
         <v>243</v>
       </c>
-      <c r="D194" s="7" t="s">
+      <c r="D194" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="E194" s="7" t="s">
+      <c r="E194" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="F194" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G194" s="2" t="s">
+      <c r="F194" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G194" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="H194" s="8" t="s">
+      <c r="H194" s="7" t="s">
         <v>245</v>
       </c>
     </row>
@@ -4186,28 +4186,28 @@
       <c r="H197" s="4"/>
     </row>
     <row r="198" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A198" s="6" t="s">
+      <c r="A198" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B198" s="2" t="s">
+      <c r="B198" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C198" s="5" t="s">
+      <c r="C198" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="D198" s="7" t="s">
+      <c r="D198" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="E198" s="7" t="s">
+      <c r="E198" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="F198" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G198" s="2" t="s">
+      <c r="F198" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G198" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H198" s="8" t="s">
+      <c r="H198" s="7" t="s">
         <v>249</v>
       </c>
     </row>
@@ -4243,6 +4243,382 @@
     </row>
   </sheetData>
   <mergeCells count="400">
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="C154:C157"/>
+    <mergeCell ref="C98:C101"/>
+    <mergeCell ref="E102:E105"/>
+    <mergeCell ref="G102:G105"/>
+    <mergeCell ref="A162:A165"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="C162:C165"/>
+    <mergeCell ref="B130:B133"/>
+    <mergeCell ref="D46:D49"/>
+    <mergeCell ref="A126:A129"/>
+    <mergeCell ref="G142:G145"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A158:A161"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="G166:G169"/>
+    <mergeCell ref="D150:D153"/>
+    <mergeCell ref="F150:F153"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="F94:F97"/>
+    <mergeCell ref="G26:G29"/>
+    <mergeCell ref="C82:C85"/>
+    <mergeCell ref="D102:D105"/>
+    <mergeCell ref="H158:H161"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="E50:E53"/>
+    <mergeCell ref="G50:G53"/>
+    <mergeCell ref="C86:C89"/>
+    <mergeCell ref="D54:D57"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="E150:E153"/>
+    <mergeCell ref="H166:H169"/>
+    <mergeCell ref="H82:H85"/>
+    <mergeCell ref="H118:H121"/>
+    <mergeCell ref="H26:H29"/>
+    <mergeCell ref="H38:H41"/>
+    <mergeCell ref="H130:H133"/>
+    <mergeCell ref="H138:H141"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="A182:A185"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="F34:F37"/>
+    <mergeCell ref="F178:F181"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="H94:H97"/>
+    <mergeCell ref="C114:C117"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="E170:E173"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="F102:F105"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="C70:C73"/>
+    <mergeCell ref="C106:C109"/>
+    <mergeCell ref="C178:C181"/>
+    <mergeCell ref="E178:E181"/>
+    <mergeCell ref="D62:D65"/>
+    <mergeCell ref="F62:F65"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="H90:H93"/>
+    <mergeCell ref="G118:G121"/>
+    <mergeCell ref="B198:B201"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A130:A133"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="F166:F169"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="E58:E61"/>
+    <mergeCell ref="D186:D189"/>
+    <mergeCell ref="B82:B85"/>
+    <mergeCell ref="F90:F93"/>
+    <mergeCell ref="E118:E121"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="E166:E169"/>
+    <mergeCell ref="F50:F53"/>
+    <mergeCell ref="A186:A189"/>
+    <mergeCell ref="C186:C189"/>
+    <mergeCell ref="D194:D197"/>
+    <mergeCell ref="F194:F197"/>
+    <mergeCell ref="A198:A201"/>
+    <mergeCell ref="B186:B189"/>
+    <mergeCell ref="A174:A177"/>
+    <mergeCell ref="G182:G185"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="D58:D61"/>
+    <mergeCell ref="F58:F61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A122:A125"/>
+    <mergeCell ref="C122:C125"/>
+    <mergeCell ref="C78:C81"/>
+    <mergeCell ref="G134:G137"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="F118:F121"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="E174:E177"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="F74:F77"/>
+    <mergeCell ref="E42:E45"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="B170:B173"/>
+    <mergeCell ref="D170:D173"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="F138:F141"/>
+    <mergeCell ref="C142:C145"/>
+    <mergeCell ref="G2:G5"/>
+    <mergeCell ref="A138:A141"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="G10:G13"/>
+    <mergeCell ref="G66:G69"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="D70:D73"/>
+    <mergeCell ref="F70:F73"/>
+    <mergeCell ref="D134:D137"/>
+    <mergeCell ref="F134:F137"/>
+    <mergeCell ref="G74:G77"/>
+    <mergeCell ref="F42:F45"/>
+    <mergeCell ref="B78:B81"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="D78:D81"/>
+    <mergeCell ref="G138:G141"/>
+    <mergeCell ref="E26:E29"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="F10:F13"/>
+    <mergeCell ref="C42:C45"/>
+    <mergeCell ref="H194:H197"/>
+    <mergeCell ref="C198:C201"/>
+    <mergeCell ref="C110:C113"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="B154:B157"/>
+    <mergeCell ref="C174:C177"/>
+    <mergeCell ref="G46:G49"/>
+    <mergeCell ref="H106:H109"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="C146:C149"/>
+    <mergeCell ref="D126:D129"/>
+    <mergeCell ref="C94:C97"/>
+    <mergeCell ref="F126:F129"/>
+    <mergeCell ref="E94:E97"/>
+    <mergeCell ref="H182:H185"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="E158:E161"/>
+    <mergeCell ref="F46:F49"/>
+    <mergeCell ref="E74:E77"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="G6:G9"/>
+    <mergeCell ref="G62:G65"/>
+    <mergeCell ref="A154:A157"/>
+    <mergeCell ref="F190:F193"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="H190:H193"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="A106:A109"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="G42:G45"/>
+    <mergeCell ref="H122:H125"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="E126:E129"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="E190:E193"/>
+    <mergeCell ref="D158:D161"/>
+    <mergeCell ref="G190:G193"/>
+    <mergeCell ref="H74:H77"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="H46:H49"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="G14:G17"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="H198:H201"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="G90:G93"/>
+    <mergeCell ref="D94:D97"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="A170:A173"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="C170:C173"/>
+    <mergeCell ref="F158:F161"/>
+    <mergeCell ref="G178:G181"/>
+    <mergeCell ref="H54:H57"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="D174:D177"/>
+    <mergeCell ref="F174:F177"/>
+    <mergeCell ref="A178:A181"/>
+    <mergeCell ref="D166:D169"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="H154:H157"/>
+    <mergeCell ref="B194:B197"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="F6:F9"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="G162:G165"/>
+    <mergeCell ref="C150:C153"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="G22:G25"/>
+    <mergeCell ref="E134:E137"/>
+    <mergeCell ref="F54:F57"/>
+    <mergeCell ref="C158:C161"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="E38:E41"/>
+    <mergeCell ref="G38:G41"/>
+    <mergeCell ref="G98:G101"/>
+    <mergeCell ref="B118:B121"/>
+    <mergeCell ref="C102:C105"/>
+    <mergeCell ref="E130:E133"/>
+    <mergeCell ref="G130:G133"/>
+    <mergeCell ref="B134:B137"/>
+    <mergeCell ref="E162:E165"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="F130:F133"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="H62:H65"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="F98:F101"/>
+    <mergeCell ref="E66:E69"/>
+    <mergeCell ref="D50:D53"/>
+    <mergeCell ref="G86:G89"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="F22:F25"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="F38:F41"/>
+    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="H42:H45"/>
+    <mergeCell ref="A194:A197"/>
+    <mergeCell ref="E54:E57"/>
+    <mergeCell ref="H86:H89"/>
+    <mergeCell ref="G54:G57"/>
+    <mergeCell ref="G114:G117"/>
+    <mergeCell ref="D118:D121"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="D182:D185"/>
+    <mergeCell ref="D38:D41"/>
+    <mergeCell ref="F182:F185"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="C74:C77"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="F162:F165"/>
+    <mergeCell ref="H162:H165"/>
+    <mergeCell ref="C166:C169"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="A118:A121"/>
+    <mergeCell ref="F114:F117"/>
+    <mergeCell ref="H114:H117"/>
+    <mergeCell ref="C118:C121"/>
+    <mergeCell ref="H70:H73"/>
+    <mergeCell ref="D66:D69"/>
+    <mergeCell ref="F66:F69"/>
+    <mergeCell ref="C194:C197"/>
+    <mergeCell ref="G110:G113"/>
+    <mergeCell ref="H150:H153"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="B150:B153"/>
+    <mergeCell ref="B190:B193"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="D190:D193"/>
+    <mergeCell ref="E82:E85"/>
+    <mergeCell ref="G82:G85"/>
+    <mergeCell ref="H102:H105"/>
+    <mergeCell ref="G146:G149"/>
+    <mergeCell ref="D122:D125"/>
+    <mergeCell ref="C90:C93"/>
+    <mergeCell ref="F122:F125"/>
+    <mergeCell ref="H178:H181"/>
+    <mergeCell ref="C182:C185"/>
+    <mergeCell ref="E182:E185"/>
+    <mergeCell ref="G70:G73"/>
+    <mergeCell ref="G58:G61"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="H58:H61"/>
+    <mergeCell ref="G186:G189"/>
+    <mergeCell ref="A190:A193"/>
+    <mergeCell ref="F186:F189"/>
+    <mergeCell ref="C190:C193"/>
+    <mergeCell ref="D74:D77"/>
+    <mergeCell ref="B138:B141"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="A142:A145"/>
+    <mergeCell ref="C14:C17"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="C134:C137"/>
+    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="C138:C141"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="B174:B177"/>
+    <mergeCell ref="A82:A85"/>
+    <mergeCell ref="E106:E109"/>
+    <mergeCell ref="D198:D201"/>
+    <mergeCell ref="F198:F201"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="E90:E93"/>
+    <mergeCell ref="F110:F113"/>
+    <mergeCell ref="H110:H113"/>
+    <mergeCell ref="B166:B169"/>
+    <mergeCell ref="E154:E157"/>
+    <mergeCell ref="G154:G157"/>
+    <mergeCell ref="B158:B161"/>
+    <mergeCell ref="H174:H177"/>
+    <mergeCell ref="A150:A153"/>
+    <mergeCell ref="H186:H189"/>
+    <mergeCell ref="D82:D85"/>
+    <mergeCell ref="F82:F85"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="F146:F149"/>
+    <mergeCell ref="H146:H149"/>
+    <mergeCell ref="G126:G129"/>
+    <mergeCell ref="E122:E125"/>
+    <mergeCell ref="G122:G125"/>
+    <mergeCell ref="E78:E81"/>
+    <mergeCell ref="G78:G81"/>
+    <mergeCell ref="H134:H137"/>
+    <mergeCell ref="G106:G109"/>
+    <mergeCell ref="E198:E201"/>
+    <mergeCell ref="G198:G201"/>
+    <mergeCell ref="G170:G173"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="H98:H101"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="D154:D157"/>
+    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="G174:G177"/>
+    <mergeCell ref="E194:E197"/>
+    <mergeCell ref="G194:G197"/>
+    <mergeCell ref="B182:B185"/>
+    <mergeCell ref="D162:D165"/>
+    <mergeCell ref="C130:C133"/>
+    <mergeCell ref="F106:F109"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="D114:D117"/>
+    <mergeCell ref="F170:F173"/>
+    <mergeCell ref="H170:H173"/>
+    <mergeCell ref="C6:C9"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="E46:E49"/>
     <mergeCell ref="D106:D109"/>
@@ -4267,382 +4643,6 @@
     <mergeCell ref="E34:E37"/>
     <mergeCell ref="G34:G37"/>
     <mergeCell ref="G30:G33"/>
-    <mergeCell ref="H134:H137"/>
-    <mergeCell ref="G106:G109"/>
-    <mergeCell ref="E198:E201"/>
-    <mergeCell ref="G198:G201"/>
-    <mergeCell ref="G170:G173"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="H6:H9"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="H98:H101"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="D154:D157"/>
-    <mergeCell ref="F154:F157"/>
-    <mergeCell ref="G174:G177"/>
-    <mergeCell ref="E194:E197"/>
-    <mergeCell ref="G194:G197"/>
-    <mergeCell ref="B182:B185"/>
-    <mergeCell ref="D162:D165"/>
-    <mergeCell ref="C130:C133"/>
-    <mergeCell ref="F106:F109"/>
-    <mergeCell ref="B114:B117"/>
-    <mergeCell ref="D114:D117"/>
-    <mergeCell ref="F170:F173"/>
-    <mergeCell ref="H170:H173"/>
-    <mergeCell ref="C6:C9"/>
-    <mergeCell ref="D198:D201"/>
-    <mergeCell ref="F198:F201"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="E90:E93"/>
-    <mergeCell ref="F110:F113"/>
-    <mergeCell ref="H110:H113"/>
-    <mergeCell ref="B166:B169"/>
-    <mergeCell ref="E154:E157"/>
-    <mergeCell ref="G154:G157"/>
-    <mergeCell ref="B158:B161"/>
-    <mergeCell ref="H174:H177"/>
-    <mergeCell ref="A150:A153"/>
-    <mergeCell ref="H186:H189"/>
-    <mergeCell ref="D82:D85"/>
-    <mergeCell ref="F82:F85"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="A94:A97"/>
-    <mergeCell ref="F146:F149"/>
-    <mergeCell ref="H146:H149"/>
-    <mergeCell ref="G126:G129"/>
-    <mergeCell ref="E122:E125"/>
-    <mergeCell ref="G122:G125"/>
-    <mergeCell ref="E78:E81"/>
-    <mergeCell ref="G78:G81"/>
-    <mergeCell ref="A190:A193"/>
-    <mergeCell ref="F186:F189"/>
-    <mergeCell ref="C190:C193"/>
-    <mergeCell ref="D74:D77"/>
-    <mergeCell ref="B138:B141"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="C14:C17"/>
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="D26:D29"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="C134:C137"/>
-    <mergeCell ref="E186:E189"/>
-    <mergeCell ref="E30:E33"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="C138:C141"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="B174:B177"/>
-    <mergeCell ref="A82:A85"/>
-    <mergeCell ref="E106:E109"/>
-    <mergeCell ref="C194:C197"/>
-    <mergeCell ref="G110:G113"/>
-    <mergeCell ref="H150:H153"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="B150:B153"/>
-    <mergeCell ref="B190:B193"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="D190:D193"/>
-    <mergeCell ref="E82:E85"/>
-    <mergeCell ref="G82:G85"/>
-    <mergeCell ref="H102:H105"/>
-    <mergeCell ref="G146:G149"/>
-    <mergeCell ref="D122:D125"/>
-    <mergeCell ref="C90:C93"/>
-    <mergeCell ref="F122:F125"/>
-    <mergeCell ref="H178:H181"/>
-    <mergeCell ref="C182:C185"/>
-    <mergeCell ref="E182:E185"/>
-    <mergeCell ref="G70:G73"/>
-    <mergeCell ref="G58:G61"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="H58:H61"/>
-    <mergeCell ref="G186:G189"/>
-    <mergeCell ref="A194:A197"/>
-    <mergeCell ref="E54:E57"/>
-    <mergeCell ref="H86:H89"/>
-    <mergeCell ref="G54:G57"/>
-    <mergeCell ref="G114:G117"/>
-    <mergeCell ref="D118:D121"/>
-    <mergeCell ref="B126:B129"/>
-    <mergeCell ref="D182:D185"/>
-    <mergeCell ref="D38:D41"/>
-    <mergeCell ref="F182:F185"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="C74:C77"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="F162:F165"/>
-    <mergeCell ref="H162:H165"/>
-    <mergeCell ref="C166:C169"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="A118:A121"/>
-    <mergeCell ref="F114:F117"/>
-    <mergeCell ref="H114:H117"/>
-    <mergeCell ref="C118:C121"/>
-    <mergeCell ref="H70:H73"/>
-    <mergeCell ref="D66:D69"/>
-    <mergeCell ref="F66:F69"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="H62:H65"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="F98:F101"/>
-    <mergeCell ref="E66:E69"/>
-    <mergeCell ref="D50:D53"/>
-    <mergeCell ref="G86:G89"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="F22:F25"/>
-    <mergeCell ref="H22:H25"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="F38:F41"/>
-    <mergeCell ref="B74:B77"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="H10:H13"/>
-    <mergeCell ref="H42:H45"/>
-    <mergeCell ref="D6:D9"/>
-    <mergeCell ref="F6:F9"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="E62:E65"/>
-    <mergeCell ref="G162:G165"/>
-    <mergeCell ref="C150:C153"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="G22:G25"/>
-    <mergeCell ref="E134:E137"/>
-    <mergeCell ref="F54:F57"/>
-    <mergeCell ref="C158:C161"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="E38:E41"/>
-    <mergeCell ref="G38:G41"/>
-    <mergeCell ref="G98:G101"/>
-    <mergeCell ref="B118:B121"/>
-    <mergeCell ref="C102:C105"/>
-    <mergeCell ref="E130:E133"/>
-    <mergeCell ref="G130:G133"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="E162:E165"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="F130:F133"/>
-    <mergeCell ref="G14:G17"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="H198:H201"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="G90:G93"/>
-    <mergeCell ref="D94:D97"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="A170:A173"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C170:C173"/>
-    <mergeCell ref="F158:F161"/>
-    <mergeCell ref="G178:G181"/>
-    <mergeCell ref="H54:H57"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="D174:D177"/>
-    <mergeCell ref="F174:F177"/>
-    <mergeCell ref="A178:A181"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="A102:A105"/>
-    <mergeCell ref="H154:H157"/>
-    <mergeCell ref="B194:B197"/>
-    <mergeCell ref="E6:E9"/>
-    <mergeCell ref="G6:G9"/>
-    <mergeCell ref="G62:G65"/>
-    <mergeCell ref="A154:A157"/>
-    <mergeCell ref="F190:F193"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="H190:H193"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="A106:A109"/>
-    <mergeCell ref="H14:H17"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="G42:G45"/>
-    <mergeCell ref="H122:H125"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="B94:B97"/>
-    <mergeCell ref="E126:E129"/>
-    <mergeCell ref="B102:B105"/>
-    <mergeCell ref="E190:E193"/>
-    <mergeCell ref="D158:D161"/>
-    <mergeCell ref="G190:G193"/>
-    <mergeCell ref="H74:H77"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="H46:H49"/>
-    <mergeCell ref="C50:C53"/>
-    <mergeCell ref="H194:H197"/>
-    <mergeCell ref="C198:C201"/>
-    <mergeCell ref="C110:C113"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="B154:B157"/>
-    <mergeCell ref="C174:C177"/>
-    <mergeCell ref="G46:G49"/>
-    <mergeCell ref="H106:H109"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="C146:C149"/>
-    <mergeCell ref="D126:D129"/>
-    <mergeCell ref="C94:C97"/>
-    <mergeCell ref="F126:F129"/>
-    <mergeCell ref="E94:E97"/>
-    <mergeCell ref="H182:H185"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="E158:E161"/>
-    <mergeCell ref="F46:F49"/>
-    <mergeCell ref="E74:E77"/>
-    <mergeCell ref="G2:G5"/>
-    <mergeCell ref="A138:A141"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="G10:G13"/>
-    <mergeCell ref="G66:G69"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="D70:D73"/>
-    <mergeCell ref="F70:F73"/>
-    <mergeCell ref="D134:D137"/>
-    <mergeCell ref="F134:F137"/>
-    <mergeCell ref="G74:G77"/>
-    <mergeCell ref="F42:F45"/>
-    <mergeCell ref="B78:B81"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="D78:D81"/>
-    <mergeCell ref="G138:G141"/>
-    <mergeCell ref="E26:E29"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="G182:G185"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="C38:C41"/>
-    <mergeCell ref="D58:D61"/>
-    <mergeCell ref="F58:F61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A122:A125"/>
-    <mergeCell ref="C122:C125"/>
-    <mergeCell ref="C78:C81"/>
-    <mergeCell ref="G134:G137"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="F118:F121"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="E174:E177"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="F74:F77"/>
-    <mergeCell ref="E42:E45"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="B170:B173"/>
-    <mergeCell ref="D170:D173"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="F138:F141"/>
-    <mergeCell ref="C142:C145"/>
-    <mergeCell ref="B198:B201"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A130:A133"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="F166:F169"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="E58:E61"/>
-    <mergeCell ref="D186:D189"/>
-    <mergeCell ref="B82:B85"/>
-    <mergeCell ref="F90:F93"/>
-    <mergeCell ref="E118:E121"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="E166:E169"/>
-    <mergeCell ref="F50:F53"/>
-    <mergeCell ref="A186:A189"/>
-    <mergeCell ref="C186:C189"/>
-    <mergeCell ref="D194:D197"/>
-    <mergeCell ref="F194:F197"/>
-    <mergeCell ref="A198:A201"/>
-    <mergeCell ref="B186:B189"/>
-    <mergeCell ref="A174:A177"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="A182:A185"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="F34:F37"/>
-    <mergeCell ref="F178:F181"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="H2:H5"/>
-    <mergeCell ref="H94:H97"/>
-    <mergeCell ref="C114:C117"/>
-    <mergeCell ref="H66:H69"/>
-    <mergeCell ref="E170:E173"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="F102:F105"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="C70:C73"/>
-    <mergeCell ref="C106:C109"/>
-    <mergeCell ref="C178:C181"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="F62:F65"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="H90:H93"/>
-    <mergeCell ref="G118:G121"/>
-    <mergeCell ref="G166:G169"/>
-    <mergeCell ref="D150:D153"/>
-    <mergeCell ref="F150:F153"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="F94:F97"/>
-    <mergeCell ref="G26:G29"/>
-    <mergeCell ref="C82:C85"/>
-    <mergeCell ref="D102:D105"/>
-    <mergeCell ref="H158:H161"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="E50:E53"/>
-    <mergeCell ref="G50:G53"/>
-    <mergeCell ref="C86:C89"/>
-    <mergeCell ref="D54:D57"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="E150:E153"/>
-    <mergeCell ref="H166:H169"/>
-    <mergeCell ref="H82:H85"/>
-    <mergeCell ref="H118:H121"/>
-    <mergeCell ref="H26:H29"/>
-    <mergeCell ref="H38:H41"/>
-    <mergeCell ref="H130:H133"/>
-    <mergeCell ref="H138:H141"/>
-    <mergeCell ref="A134:A137"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="C154:C157"/>
-    <mergeCell ref="C98:C101"/>
-    <mergeCell ref="E102:E105"/>
-    <mergeCell ref="G102:G105"/>
-    <mergeCell ref="A162:A165"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="C162:C165"/>
-    <mergeCell ref="B130:B133"/>
-    <mergeCell ref="D46:D49"/>
-    <mergeCell ref="A126:A129"/>
-    <mergeCell ref="G142:G145"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A158:A161"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="A98:A101"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>